<commit_message>
Every RCJ disposition re-read against the 2026-09-24 pull; each builder runs the prose rule
26 existing dispositions rebuilt; each refuses an uncovered candidate and
calls rhtp_assert_disposition_prose() before writing. TN, NJ and WY gain
tier3_candidates. Findings: Louisiana's Rural Clinician Credit Bank has
awarded (53, 20 to hospitals, 5 named); NV, NE (5.3) and MI award files are
incomplete against live state pages; CA Distressed Hospital Small Grants,
TX NFP/Workplace Violence/HOPES, DE DDD rebates and MI CVI are state money
carried as RHTP. New evidence archived under recheck/2026-09-24/.
Session 63 record and CLAUDE.md current state.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019fxT82oSxjU7hDb4oJm1m7
</commit_message>
<xml_diff>
--- a/DE_year1_awardees.xlsx
+++ b/DE_year1_awardees.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
   <si>
     <t xml:space="preserve">READ_THIS_FIRST</t>
   </si>
@@ -380,6 +380,9 @@
     <t xml:space="preserve">rcj_rows</t>
   </si>
   <si>
+    <t xml:space="preserve">withdrawn_rows</t>
+  </si>
+  <si>
     <t xml:space="preserve">disposition</t>
   </si>
   <si>
@@ -392,7 +395,16 @@
     <t xml:space="preserve">REAL_AWARDS_CARRIED_AT_A_$1_PLACEHOLDER</t>
   </si>
   <si>
-    <t xml:space="preserve">RCJ carries all four, NAMED EXACTLY AS DELAWARE PRINTS THEM (site and all), at an amount of $1 each. Missouri's and Maine's placeholder mechanism: the aggregator is RIGHT about the recipients and says nothing usable about the money, so no amount check can see the defect -- EXCEPT THAT STAGE 2 ALREADY CAUGHT IT: all four carry `flag_reason = AMOUNT_IMPLAUSIBLE_LOW` in the committed record table, which is the $1 placeholder showing up as a plausibility failure four sessions before anyone read the release. These four ARE this file's rows, and the amounts come from Delaware -- which published none.</t>
+    <t xml:space="preserve">RCJ carries all 4, NAMED EXACTLY AS DELAWARE PRINTS THEM (site and all), at an amount of $1 each. Missouri's and Maine's placeholder mechanism: the aggregator is RIGHT about the recipients and says nothing usable about the money, so no amount check can see the defect -- EXCEPT THAT STAGE 2 ALREADY CAUGHT IT: every one carries `flag_reason = AMOUNT_IMPLAUSIBLE_LOW`, which is the $1 placeholder showing up as a plausibility failure. These ARE this file's rows, and the amounts come from Delaware -- which published none. ON THE 2026-09-24 PULL RCJ RE-KEYED THEM: the 4 rows first seen 2026-08-27 were WITHDRAWN and the same 4 recipients re-filed under new record ids with rewritten descriptions -- the same four awards, not new ones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtown Development Districts rebate reservations -- DSHA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT_RHTP_STATE_PROGRAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 of Delaware's 12 live Tier 3 candidates, first seen on the 2026-09-24 pull, all from DSHA's 2026-09-10 release 'Large Projects Awarded Downtown Development Districts Funding Reservations' ($3,433,344 to real-estate investors: Leroy Tice Esquire, Wilmington; Little Living Org. Inc., Georgetown; Loockerman Plaza LLC, Dover; Mach Investments LLC, Smyrna; Nas Homes LLC, Wilmington; Office Partners XIX Brandywine LLC (two projects), Wilmington; Tatnall West II LLC, Wilmington). §0.1 FAILURE MODE 1, the wrong programme, and not health care at all: DSHA's Downtown Development Districts rebate program, established 2014, funded by 'state appropriations' ('$47.4 million in state funds'), reserving rebates for commercial and residential revitalisation. The release mentions RHTP, 'Rural Health Transformation', 'federal' and 'CMS' ZERO times. It shares only a publisher (news.delaware.gov) with the school-based release. Archived: data/evidence/recheck/2026-09-24/DE/2026-09-10_de_dsha_downtown_development_districts_STATE_PROGRAM.html.</t>
   </si>
   <si>
     <t xml:space="preserve">Delaware State Housing Authority</t>
@@ -401,16 +413,16 @@
     <t xml:space="preserve">TIER_2_BUDGET_LINE</t>
   </si>
   <si>
-    <t xml:space="preserve">$11,500,000, sourced to 'DE - 2025 - Delaware RHTP Executive Budget Summary'. A budget-narrative line item, not a subaward (Oklahoma's and Connecticut's tier defect). DHSS's programme page carries no housing initiative among its fifteen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Red Health Center, Inc.</t>
+    <t xml:space="preserve">$11,500,000, sourced to 'DE - 2025 - Delaware RHTP Executive Budget Summary'. A budget-narrative line item, not a subaward (Oklahoma's and Connecticut's tier defect): RCJ's own description is the renovation of two state-owned buildings as Rural Hope Centers, which is DHSS's 'Hope Centers' initiative -- one of its fifteen, with a Year 1 budget and no recipient named (de_year1_status.csv).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Red Health Center, Inc. (WITHDRAWN BY RCJ)</t>
   </si>
   <si>
     <t xml:space="preserve">NOT_RHTP_FEDERAL_PROVENANCE_ALREADY_QUARANTINED</t>
   </si>
   <si>
-    <t xml:space="preserve">$250,000, sourced to 'FY 2025: HRSA's Rural Health Grants Delaware Fact Sheet'. THE ORIGINAL §6.2 FINDING, from Stage 0: a different FEDERAL programme's money on a HRSA document, which is why the provenance filter exists at all. It is already QUARANTINED in the record table with `PROVENANCE_MISMATCH`, which is why the 50-state survey counts FIVE Delaware candidates and the record table holds SIX -- the survey counts PASS and FLAGGED rows only. This disposition covers all six.</t>
+    <t xml:space="preserve">RCJ WITHDREW THIS ROW ON THE 2026-09-24 PULL; 0 live. It was $250,000, sourced to 'FY 2025: HRSA's Rural Health Grants Delaware Fact Sheet'. THE ORIGINAL §6.2 FINDING, from Stage 0: a different FEDERAL programme's money on a HRSA document, which is why the provenance filter exists at all; it was QUARANTINED with `PROVENANCE_MISMATCH`. Kept, not deleted: withdrawal is a fact about the aggregator, and if RCJ re-files it this group describes it again.</t>
   </si>
 </sst>
 </file>
@@ -1732,10 +1744,11 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="33.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="58.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="47.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="250.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="47.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="250.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1754,56 +1767,88 @@
       <c r="E1" s="1" t="s">
         <v>122</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" t="n">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>124</v>
+      <c r="D2" t="n">
+        <v>4</v>
       </c>
       <c r="E2" t="s">
         <v>125</v>
       </c>
+      <c r="F2" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>127</v>
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
       </c>
       <c r="E3" t="s">
         <v>128</v>
       </c>
+      <c r="F3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
-        <v>130</v>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
       <c r="E4" t="s">
         <v>131</v>
+      </c>
+      <c r="F4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F5" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>